<commit_message>
Workbook edits from 2026-09 (wealth CALC + ops blue cells), validated with make check
</commit_message>
<xml_diff>
--- a/data/command-center.xlsx
+++ b/data/command-center.xlsx
@@ -30,1440 +30,1470 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="478">
-  <si>
-    <t xml:space="preserve">◆ BALANCES — Bank &amp; Investment Accounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update balances weekly. Blue cells = your input. Black cells = formulas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Institution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balance (BRL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balance (USD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Updated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Banco Inter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conta 662710-2 · R$18,922.07 disp + R$12.60 bloq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mercado Pago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extrato MP PDF 01-12/Jul/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BB Brasil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rende Fácil balance not in export</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL LIQUID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ INVESTMENTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Instrument</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL Equiv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IB Net Deposits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brokerage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan-Jun 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEPLOYED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto: FX_OPS IB Deposit sum - IB Withdraw sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fundos BRL — Topázio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fund</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May-Jun 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto: FX_OPS Fund Deposit sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL INVESTMENTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EST. NET WORTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEGEND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🔵 Blue text = your input (edit these cells)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚫ Black text = formula (do not edit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🟢 Green text = cross-sheet formula (auto-calculated from FX_OPS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🟡 Yellow background = input cells</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ FX OPERATIONS — BCB Câmbio Register</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Append one row per BCB câmbio operation. Source: BCB Câmbio PDF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Destination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CCY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FCY Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Banco Topázio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Interactive Brokers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IB Deposit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91992 IB deposit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USA - Own Account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outbound</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67995 Self-transfer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67995 via Inter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wise Brasil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UK - Eduardo Giovannini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67995 Wise UK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91992 IB via Wise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fundos investimento BRL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fund Deposit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67043 Fund capital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USA → Eduardo Forster Giovannini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inbound</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72629 Inbound from USA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ouribank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inbound payment order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72629 Inbound payment order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IB Withdraw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91992 IB withdrawal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ DIRECTION SUMMARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FCY Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avg Rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ TRANSACTIONS — MP Faturas Card Statement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paste new transactions when each fatura closes. 146 entries Jan-Jun 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fatura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merchant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value (BRL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">International</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFD*PIZZA NOW INTERMARES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delivery/iFood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Não</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPENAI *CHATGPT SUBSCR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IA/Tecnologia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APPLE.COM/BILL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assinatura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFD*34531468 EDWIN LEI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANUS AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DL*Starlink Braz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP*LOTERIASONLINEU1AQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loteria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IFD*FORMAGGIO RESTAURANTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP*LOTERIASONLINE542V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEMSQZY* PINEAPPLE-APP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLAUDE.AI SUBSCRIPTION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RAYCAST.COM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DESKTOP COMMANDER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP*LOTERIASONLINEM4UQ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP*LOTERIASONLINEYY48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MERCADOLIVRE*3PRODUTOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compras/ML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANTHROPIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP*LOTERIASONLINEO4M4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DL *Starlink Brazil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-02-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MERCADOLIVRE*7PRODUTOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GITHUB, INC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAN AIRLINE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viagem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OPENROUTER, INC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STARLINK INTERNET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROK XAI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CURSOR AI POWERED IDE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MICROSOFT*STORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLOUDFLARE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PERPLEXITY.AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DL*GOOGLE YouTub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONTA VIVO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Telecomunicações</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ SUMMARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TX COUNT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠ This contains a representative 59-tx subset. Paste full 146-tx MP Faturas data to replace.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ SUBSCRIPTIONS — 15 Services Tracked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update decisions and status. Renewal dates from Apple Subscriptions export.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly BRL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dup Risk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renewal Date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">automacao.giovannini@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - General/Coding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HIGH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANCEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cadastros.online1979@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ChatGPT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">giovannini.eduardo@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - General Assistant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEDIUM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEEP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - General/Workspace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVIEW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cadastro.giovannini@gmail.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - Agent/Credits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNKNOWN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cursor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - Coding Assistant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desktop Commander</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unlimited</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - Desktop Automation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filmora9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creative/Productivity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperGrok</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - General/Media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iCloud+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200 GB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cloud/Storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Microsoft 365</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Personal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Productivity/Cloud</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027-06-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NordVPN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Security/VPN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perplexity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pro Mac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI - Research</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TuneIn Radio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Premium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entertainment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ DECISION SUMMARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEEP total/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANCEL savings/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVIEW total/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANCEL savings/yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL STACK/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ PIX — Banco Inter Cash Bridge · Account 6627102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paste from Inter extrato. PIX + Câmbio + IOF movements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counterpart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIX Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IOF Amount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIX In</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduardo Forster Giovannini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduardo F Giovannini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-06-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIX Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduardo Silva Dos Santos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-05-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moacir Jose De Morais Filho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucas Rique Chaves Bezerra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sbct Tech Solutions Llc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduardo Giovannini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wise Brasil Corretora De Cambio Ltda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Câmbio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Envio - remessa internacional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IOF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IOF - Operação de câmbio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gloria Raquel M C Nobrega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mag Administracao De Negocios Ltda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-04-24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jose Periclis De Sousa Da Costa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iago Kevyn Santos Moura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-03-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mercado Pago Instituicao De Pagamento Ltda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net PIX Flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Câmbio Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total IOF Paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ REPOS — Git Repository Health · ~/Documents/GitHub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update via rescan-repos.zsh output. Currently 2 repos on iMac M3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Branch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dirty Files</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Commit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Days Since</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remote</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Language</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk Score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">financas-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dirty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">main</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">github.com/AUTOGIO/financas-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Python</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary finance workspace · command-center source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MacHealthOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">github.com/AUTOGIO/MacHealthOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swift</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mac system health monitoring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ STATUS SUMMARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Repos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dirty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Broken</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Add more repos as you clone them to the iMac. Run rescan-repos.zsh to auto-populate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ PROJECTS — Operational Status Board</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manual update. One row per active project. This is NOT automated — it is your 2-min status board.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current Focus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Next Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Touched</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command Center build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complete xlsx + html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iMac M3 setup from zero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Continue system configuration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Global Retirement ETF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paused</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portfolio architecture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waiting for iMac setup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clone repo to iMac when ready</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IBKR-Excel-Bridge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IB → Excel snapshots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs TWS on iMac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Install TWS, clone repo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PersonalLifeOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SwiftUI habits/schedule</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs clean Xcode build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verify build on MBA, then clone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTOGIO_PIOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UniFi/Starlink health</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WAN stability gate reset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-run WAN gate when on iMac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ COUNTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ CONFIG — Alert Thresholds &amp; Parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit values to change what triggers alerts in the Command Center.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liquidity Floor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if TOTAL LIQUID &lt; this value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly Burn Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if card spend in any month exceeds this</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subscription Stack Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if total KEEP subscriptions &gt; this</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repo Staleness Days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Risk score +5 if repo has no commit in this many days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Rate Low Alert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL/USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if any FX op below this rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Rate High Alert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if any FX op above this rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel Savings Target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expected monthly savings from CANCEL queue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renewal Warning Days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert when a subscription renewal is within this many days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Stale Days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alert if active project not touched in this many days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net Worth Currency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All amounts denominated in BRL unless marked USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Report Period</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H1 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Owner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPF redacted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ MONTHLY — Cash Flow Summary · Jan–Jun 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One row per month. Card from TRANSACTIONS, PIX from PIX tab, FX from FX_OPS. Update when new month closes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Card Spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Txs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX In</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net Flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL H1 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AVG/MONTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ MoM CHANGES — Card Spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prior Month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MoM %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ CATEGORIES — Card Spend Breakdown · H1 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sorted largest to smallest. Update when full transaction data changes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total (R$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% of Card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avg/Month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">💡 Discretionary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠ Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">❓ Unknown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">✅ Essential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transporte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ BY CLASSIFICATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">◆ ALERTS — Risk &amp; Action Register · Cross-Domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full alert register. Sources: finance, subscriptions, repos, projects. Update status as resolved.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRL Exposure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recommended Action</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRITICAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subscriptions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CANCEL queue: Claude x2 (R$184/mo) + Grok (R$149.90/mo) + TuneIn (R$31.90/mo) = R$365.80/mo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cancel all 4 before next billing. Apple Subscriptions + app accounts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FX Reconciliation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$652,789 sent to USA Own Account (67995). 19 ops Jan-Jun. Validate USD balances vs BCB.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pull USD account statement. Reconcile each BCB op against balance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sub Stack Bloat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 services in REVIEW. Annual exposure ~R$7,763. Manus credits uncontrolled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audit each REVIEW service. Decide KEEP/CANCEL. Target: eliminate ≥3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liquidity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100% liquid in 2 digital banks (Inter + MP = R$23,197). BB balance R$0. Below R$30k target.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maintain R$30k+ buffer. Distribute across BB Rende Fácil + Inter.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IOF + FX Cost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$3,475 IOF paid on Inter FX. Compare rates across Wise / Topázio / BB.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Review IOF rate per op. Compare institutions for next transfers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IB Withdrawal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$19,196 IB withdrawal via Wise Jun/2026. Destination unconfirmed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm destination. Check Inter + IB statements.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lottery/Gambling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$6,455 Loteria on MP card (39 txs). No budget cap. Avg R$1,076/mo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set monthly Loteria limit R$500. Remove card if exceeded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI/Tech Overlap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$6,624 via card on IA/Tech (37 txs). Likely duplicates subscription stack.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross-match card IA charges vs sub list. Consolidate billing method.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travel/Viagem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$9,037 travel charges (LAN Airlines Mar/2026). Business vs personal unclassified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classify: business vs personal. Flag deductible items.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ML Volume</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$31,570 Mercado Livre purchases. Strong Home Office + CPAP pattern. No tags.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tag each purchase: CAPEX / HEALTH / CONSUMABLE for tax tracking.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multiple Wise ops (IB deposits + UK transfers). Ensure BACEN reporting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm BACEN reporting compliance. Keep KYC current.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SBCT Tech Solutions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$45,000 PIX Out to SBCT Tech Solutions LLC (USA) via Inter May/2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm nature: service invoice? investment? Ensure documentation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="488">
+  <si>
+    <t>◆ BALANCES — Bank &amp;amp; Investment Accounts</t>
+  </si>
+  <si>
+    <t>Update balances weekly. Blue cells = your input. Black cells = formulas.</t>
+  </si>
+  <si>
+    <t>Institution</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Balance (BRL)</t>
+  </si>
+  <si>
+    <t>Balance (USD)</t>
+  </si>
+  <si>
+    <t>Last Updated</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Banco Inter</t>
+  </si>
+  <si>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>CONFIRMED</t>
+  </si>
+  <si>
+    <t>Conta 662710-2 · R$18,922.07 disp + R$12.60 bloq</t>
+  </si>
+  <si>
+    <t>Mercado Pago</t>
+  </si>
+  <si>
+    <t>2026-07-12</t>
+  </si>
+  <si>
+    <t>Extrato MP PDF 01-12/Jul/2026</t>
+  </si>
+  <si>
+    <t>BB Brasil</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>Rende Fácil balance not in export</t>
+  </si>
+  <si>
+    <t>TOTAL LIQUID</t>
+  </si>
+  <si>
+    <t>◆ INVESTMENTS</t>
+  </si>
+  <si>
+    <t>Instrument</t>
+  </si>
+  <si>
+    <t>BRL Equiv</t>
+  </si>
+  <si>
+    <t>USD Amount</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>IB Net Deposits</t>
+  </si>
+  <si>
+    <t>Brokerage</t>
+  </si>
+  <si>
+    <t>Jan-Jun 2026</t>
+  </si>
+  <si>
+    <t>DEPLOYED</t>
+  </si>
+  <si>
+    <t>Auto: FX_OPS IB Deposit sum - IB Withdraw sum</t>
+  </si>
+  <si>
+    <t>Fundos BRL — Topázio</t>
+  </si>
+  <si>
+    <t>Fund</t>
+  </si>
+  <si>
+    <t>May-Jun 2026</t>
+  </si>
+  <si>
+    <t>Auto: FX_OPS Fund Deposit sum</t>
+  </si>
+  <si>
+    <t>TOTAL INVESTMENTS</t>
+  </si>
+  <si>
+    <t>EST. NET WORTH</t>
+  </si>
+  <si>
+    <t>LEGEND</t>
+  </si>
+  <si>
+    <t>🔵 Blue text = your input (edit these cells)</t>
+  </si>
+  <si>
+    <t>⚫ Black text = formula (do not edit)</t>
+  </si>
+  <si>
+    <t>🟢 Green text = cross-sheet formula (auto-calculated from FX_OPS)</t>
+  </si>
+  <si>
+    <t>🟡 Yellow background = input cells</t>
+  </si>
+  <si>
+    <t>◆ FX OPERATIONS — BCB Câmbio Register</t>
+  </si>
+  <si>
+    <t>Append one row per BCB câmbio operation. Source: BCB Câmbio PDF.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>CCY</t>
+  </si>
+  <si>
+    <t>FCY Amount</t>
+  </si>
+  <si>
+    <t>BRL Amount</t>
+  </si>
+  <si>
+    <t>FX Rate</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
+  <si>
+    <t>Nature</t>
+  </si>
+  <si>
+    <t>2026-01-26</t>
+  </si>
+  <si>
+    <t>Banco Topázio</t>
+  </si>
+  <si>
+    <t>Interactive Brokers</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>IB Deposit</t>
+  </si>
+  <si>
+    <t>91992 IB deposit</t>
+  </si>
+  <si>
+    <t>2026-01-27</t>
+  </si>
+  <si>
+    <t>USA - Own Account</t>
+  </si>
+  <si>
+    <t>Outbound</t>
+  </si>
+  <si>
+    <t>67995 Self-transfer</t>
+  </si>
+  <si>
+    <t>2026-01-30</t>
+  </si>
+  <si>
+    <t>2026-02-09</t>
+  </si>
+  <si>
+    <t>2026-02-11</t>
+  </si>
+  <si>
+    <t>2026-03-03</t>
+  </si>
+  <si>
+    <t>2026-03-13</t>
+  </si>
+  <si>
+    <t>2026-03-18</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>67995 via Inter</t>
+  </si>
+  <si>
+    <t>2026-05-11</t>
+  </si>
+  <si>
+    <t>2026-05-15</t>
+  </si>
+  <si>
+    <t>Wise Brasil</t>
+  </si>
+  <si>
+    <t>UK - Eduardo Giovannini</t>
+  </si>
+  <si>
+    <t>67995 Wise UK</t>
+  </si>
+  <si>
+    <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>91992 IB via Wise</t>
+  </si>
+  <si>
+    <t>2026-05-19</t>
+  </si>
+  <si>
+    <t>2026-05-20</t>
+  </si>
+  <si>
+    <t>2026-05-22</t>
+  </si>
+  <si>
+    <t>Fundos investimento BRL</t>
+  </si>
+  <si>
+    <t>BRL</t>
+  </si>
+  <si>
+    <t>Fund Deposit</t>
+  </si>
+  <si>
+    <t>67043 Fund capital</t>
+  </si>
+  <si>
+    <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>USA → Eduardo Forster Giovannini</t>
+  </si>
+  <si>
+    <t>Inbound</t>
+  </si>
+  <si>
+    <t>72629 Inbound from USA</t>
+  </si>
+  <si>
+    <t>2026-06-16</t>
+  </si>
+  <si>
+    <t>Ouribank</t>
+  </si>
+  <si>
+    <t>Inbound payment order</t>
+  </si>
+  <si>
+    <t>72629 Inbound payment order</t>
+  </si>
+  <si>
+    <t>2026-06-19</t>
+  </si>
+  <si>
+    <t>2026-06-22</t>
+  </si>
+  <si>
+    <t>2026-06-26</t>
+  </si>
+  <si>
+    <t>IB Withdraw</t>
+  </si>
+  <si>
+    <t>91992 IB withdrawal</t>
+  </si>
+  <si>
+    <t>◆ DIRECTION SUMMARY</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>BRL Total</t>
+  </si>
+  <si>
+    <t>FCY Total</t>
+  </si>
+  <si>
+    <t>Avg Rate</t>
+  </si>
+  <si>
+    <t>◆ TRANSACTIONS — MP Faturas Card Statement</t>
+  </si>
+  <si>
+    <t>Paste new transactions when each fatura closes. 146 entries Jan-Jun 2026.</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Fatura</t>
+  </si>
+  <si>
+    <t>Merchant</t>
+  </si>
+  <si>
+    <t>Value (BRL)</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>International</t>
+  </si>
+  <si>
+    <t>2026-01-06</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>IFD*PIZZA NOW INTERMARES</t>
+  </si>
+  <si>
+    <t>Delivery/iFood</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>2026-01-08</t>
+  </si>
+  <si>
+    <t>OPENAI *CHATGPT SUBSCR</t>
+  </si>
+  <si>
+    <t>IA/Tecnologia</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>APPLE.COM/BILL</t>
+  </si>
+  <si>
+    <t>Assinatura</t>
+  </si>
+  <si>
+    <t>2026-01-10</t>
+  </si>
+  <si>
+    <t>IFD*34531468 EDWIN LEI</t>
+  </si>
+  <si>
+    <t>2026-01-14</t>
+  </si>
+  <si>
+    <t>MANUS AI</t>
+  </si>
+  <si>
+    <t>2026-01-15</t>
+  </si>
+  <si>
+    <t>DL*Starlink Braz</t>
+  </si>
+  <si>
+    <t>Internet</t>
+  </si>
+  <si>
+    <t>2026-01-16</t>
+  </si>
+  <si>
+    <t>MP*LOTERIASONLINEU1AQ</t>
+  </si>
+  <si>
+    <t>Loteria</t>
+  </si>
+  <si>
+    <t>IFD*FORMAGGIO RESTAURANTE</t>
+  </si>
+  <si>
+    <t>2026-01-17</t>
+  </si>
+  <si>
+    <t>MP*LOTERIASONLINE542V</t>
+  </si>
+  <si>
+    <t>2026-01-19</t>
+  </si>
+  <si>
+    <t>LEMSQZY* PINEAPPLE-APP</t>
+  </si>
+  <si>
+    <t>2026-01-21</t>
+  </si>
+  <si>
+    <t>CLAUDE.AI SUBSCRIPTION</t>
+  </si>
+  <si>
+    <t>RAYCAST.COM</t>
+  </si>
+  <si>
+    <t>Outros</t>
+  </si>
+  <si>
+    <t>2026-01-28</t>
+  </si>
+  <si>
+    <t>2026-02-03</t>
+  </si>
+  <si>
+    <t>DESKTOP COMMANDER</t>
+  </si>
+  <si>
+    <t>2026-02-04</t>
+  </si>
+  <si>
+    <t>MP*LOTERIASONLINEM4UQ</t>
+  </si>
+  <si>
+    <t>2026-02-05</t>
+  </si>
+  <si>
+    <t>MP*LOTERIASONLINEYY48</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>MERCADOLIVRE*3PRODUTOS</t>
+  </si>
+  <si>
+    <t>Compras/ML</t>
+  </si>
+  <si>
+    <t>2026-02-14</t>
+  </si>
+  <si>
+    <t>ANTHROPIC</t>
+  </si>
+  <si>
+    <t>MP*LOTERIASONLINEO4M4</t>
+  </si>
+  <si>
+    <t>2026-02-16</t>
+  </si>
+  <si>
+    <t>DL *Starlink Brazil</t>
+  </si>
+  <si>
+    <t>2026-02-17</t>
+  </si>
+  <si>
+    <t>2026-02-21</t>
+  </si>
+  <si>
+    <t>2026-03-05</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-03-08</t>
+  </si>
+  <si>
+    <t>MERCADOLIVRE*7PRODUTOS</t>
+  </si>
+  <si>
+    <t>GITHUB, INC.</t>
+  </si>
+  <si>
+    <t>2026-03-10</t>
+  </si>
+  <si>
+    <t>LAN AIRLINE</t>
+  </si>
+  <si>
+    <t>Viagem</t>
+  </si>
+  <si>
+    <t>OPENROUTER, INC</t>
+  </si>
+  <si>
+    <t>2026-03-14</t>
+  </si>
+  <si>
+    <t>STARLINK INTERNET</t>
+  </si>
+  <si>
+    <t>2026-03-17</t>
+  </si>
+  <si>
+    <t>2026-03-21</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>GROK XAI</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>CURSOR AI POWERED IDE</t>
+  </si>
+  <si>
+    <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>MICROSOFT*STORE</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>CLOUDFLARE</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>PERPLEXITY.AI</t>
+  </si>
+  <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>2026-05-03</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-05-08</t>
+  </si>
+  <si>
+    <t>2026-05-17</t>
+  </si>
+  <si>
+    <t>DL*GOOGLE YouTub</t>
+  </si>
+  <si>
+    <t>2026-05-30</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>2026-06-03</t>
+  </si>
+  <si>
+    <t>CONTA VIVO</t>
+  </si>
+  <si>
+    <t>Telecomunicações</t>
+  </si>
+  <si>
+    <t>2026-06-04</t>
+  </si>
+  <si>
+    <t>◆ SUMMARY</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>TX COUNT</t>
+  </si>
+  <si>
+    <t>⚠ This contains a representative 59-tx subset. Paste full 146-tx MP Faturas data to replace.</t>
+  </si>
+  <si>
+    <t>◆ SUBSCRIPTIONS — 15 Services Tracked</t>
+  </si>
+  <si>
+    <t>Update decisions and status. Renewal dates from Apple Subscriptions export.</t>
+  </si>
+  <si>
+    <t>Service</t>
+  </si>
+  <si>
+    <t>Plan</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Monthly BRL</t>
+  </si>
+  <si>
+    <t>Dup Risk</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Renewal Date</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>Pro</t>
+  </si>
+  <si>
+    <t>automacao.giovannini@gmail.com</t>
+  </si>
+  <si>
+    <t>AI - General/Coding</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>CANCEL</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>cadastros.online1979@gmail.com</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Plus</t>
+  </si>
+  <si>
+    <t>giovannini.eduardo@gmail.com</t>
+  </si>
+  <si>
+    <t>AI - General Assistant</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>KEEP</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>AI - General/Workspace</t>
+  </si>
+  <si>
+    <t>REVIEW</t>
+  </si>
+  <si>
+    <t>Manus</t>
+  </si>
+  <si>
+    <t>Credits</t>
+  </si>
+  <si>
+    <t>cadastro.giovannini@gmail.com</t>
+  </si>
+  <si>
+    <t>UNK</t>
+  </si>
+  <si>
+    <t>AI - Agent/Credits</t>
+  </si>
+  <si>
+    <t>UNKNOWN</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Cursor</t>
+  </si>
+  <si>
+    <t>AI - Coding Assistant</t>
+  </si>
+  <si>
+    <t>Desktop Commander</t>
+  </si>
+  <si>
+    <t>Unlimited</t>
+  </si>
+  <si>
+    <t>AI - Desktop Automation</t>
+  </si>
+  <si>
+    <t>Filmora9</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>Creative/Productivity</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>SuperGrok</t>
+  </si>
+  <si>
+    <t>AI - General/Media</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>iCloud+</t>
+  </si>
+  <si>
+    <t>200 GB</t>
+  </si>
+  <si>
+    <t>Cloud/Storage</t>
+  </si>
+  <si>
+    <t>2026-07-10</t>
+  </si>
+  <si>
+    <t>Microsoft 365</t>
+  </si>
+  <si>
+    <t>Personal</t>
+  </si>
+  <si>
+    <t>Productivity/Cloud</t>
+  </si>
+  <si>
+    <t>2027-06-20</t>
+  </si>
+  <si>
+    <t>NordVPN</t>
+  </si>
+  <si>
+    <t>Security/VPN</t>
+  </si>
+  <si>
+    <t>2026-10-06</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>Pro Mac</t>
+  </si>
+  <si>
+    <t>AI - Research</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>TuneIn Radio</t>
+  </si>
+  <si>
+    <t>Premium</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>2026-07-23</t>
+  </si>
+  <si>
+    <t>◆ DECISION SUMMARY</t>
+  </si>
+  <si>
+    <t>KEEP total/mo</t>
+  </si>
+  <si>
+    <t>CANCEL savings/mo</t>
+  </si>
+  <si>
+    <t>REVIEW total/mo</t>
+  </si>
+  <si>
+    <t>CANCEL savings/yr</t>
+  </si>
+  <si>
+    <t>TOTAL STACK/mo</t>
+  </si>
+  <si>
+    <t>◆ PIX — Banco Inter Cash Bridge · Account 6627102</t>
+  </si>
+  <si>
+    <t>Paste from Inter extrato. PIX + Câmbio + IOF movements.</t>
+  </si>
+  <si>
+    <t>Counterpart</t>
+  </si>
+  <si>
+    <t>PIX Amount</t>
+  </si>
+  <si>
+    <t>FX Amount</t>
+  </si>
+  <si>
+    <t>IOF Amount</t>
+  </si>
+  <si>
+    <t>2026-06-28</t>
+  </si>
+  <si>
+    <t>PIX In</t>
+  </si>
+  <si>
+    <t>Eduardo Forster Giovannini</t>
+  </si>
+  <si>
+    <t>Eduardo F Giovannini</t>
+  </si>
+  <si>
+    <t>2026-06-25</t>
+  </si>
+  <si>
+    <t>PIX Out</t>
+  </si>
+  <si>
+    <t>Eduardo Silva Dos Santos</t>
+  </si>
+  <si>
+    <t>2026-05-25</t>
+  </si>
+  <si>
+    <t>2026-05-24</t>
+  </si>
+  <si>
+    <t>Moacir Jose De Morais Filho</t>
+  </si>
+  <si>
+    <t>Lucas Rique Chaves Bezerra</t>
+  </si>
+  <si>
+    <t>Sbct Tech Solutions Llc</t>
+  </si>
+  <si>
+    <t>Eduardo Giovannini</t>
+  </si>
+  <si>
+    <t>Wise Brasil Corretora De Cambio Ltda</t>
+  </si>
+  <si>
+    <t>Câmbio</t>
+  </si>
+  <si>
+    <t>Envio - remessa internacional</t>
+  </si>
+  <si>
+    <t>IOF</t>
+  </si>
+  <si>
+    <t>IOF - Operação de câmbio</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>Gloria Raquel M C Nobrega</t>
+  </si>
+  <si>
+    <t>Mag Administracao De Negocios Ltda</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>Jose Periclis De Sousa Da Costa</t>
+  </si>
+  <si>
+    <t>2026-03-20</t>
+  </si>
+  <si>
+    <t>Iago Kevyn Santos Moura</t>
+  </si>
+  <si>
+    <t>2026-03-15</t>
+  </si>
+  <si>
+    <t>Mercado Pago Instituicao De Pagamento Ltda</t>
+  </si>
+  <si>
+    <t>Net PIX Flow</t>
+  </si>
+  <si>
+    <t>Total Câmbio Out</t>
+  </si>
+  <si>
+    <t>Total IOF Paid</t>
+  </si>
+  <si>
+    <t>◆ REPOS — Git Repository Health · ~/Documents/GitHub</t>
+  </si>
+  <si>
+    <t>Update via rescan-repos.zsh output. Currently 2 repos on iMac M3.</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Branch</t>
+  </si>
+  <si>
+    <t>Dirty Files</t>
+  </si>
+  <si>
+    <t>Last Commit</t>
+  </si>
+  <si>
+    <t>Days Since</t>
+  </si>
+  <si>
+    <t>Remote</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>Risk Score</t>
+  </si>
+  <si>
+    <t>financas-2026</t>
+  </si>
+  <si>
+    <t>dirty</t>
+  </si>
+  <si>
+    <t>main</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
+  </si>
+  <si>
+    <t>github.com/AUTOGIO/financas-2026</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>Primary finance workspace · command-center source</t>
+  </si>
+  <si>
+    <t>MacHealthOS</t>
+  </si>
+  <si>
+    <t>github.com/AUTOGIO/MacHealthOS</t>
+  </si>
+  <si>
+    <t>Swift</t>
+  </si>
+  <si>
+    <t>Mac system health monitoring</t>
+  </si>
+  <si>
+    <t>◆ STATUS SUMMARY</t>
+  </si>
+  <si>
+    <t>Total Repos</t>
+  </si>
+  <si>
+    <t>Clean</t>
+  </si>
+  <si>
+    <t>Dirty</t>
+  </si>
+  <si>
+    <t>Broken</t>
+  </si>
+  <si>
+    <t>Add more repos as you clone them to the iMac. Run rescan-repos.zsh to auto-populate.</t>
+  </si>
+  <si>
+    <t>◆ PROJECTS — Operational Status Board</t>
+  </si>
+  <si>
+    <t>Manual update. One row per active project. This is NOT automated — it is your 2-min status board.</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Current Focus</t>
+  </si>
+  <si>
+    <t>Blocker</t>
+  </si>
+  <si>
+    <t>Next Action</t>
+  </si>
+  <si>
+    <t>Last Touched</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Command Center build</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Complete xlsx + html</t>
+  </si>
+  <si>
+    <t>iMac M3 setup from zero</t>
+  </si>
+  <si>
+    <t>Continue system configuration</t>
+  </si>
+  <si>
+    <t>Global Retirement ETF</t>
+  </si>
+  <si>
+    <t>Paused</t>
+  </si>
+  <si>
+    <t>Portfolio architecture</t>
+  </si>
+  <si>
+    <t>Waiting for iMac setup</t>
+  </si>
+  <si>
+    <t>Clone repo to iMac when ready</t>
+  </si>
+  <si>
+    <t>IBKR-Excel-Bridge</t>
+  </si>
+  <si>
+    <t>IB → Excel snapshots</t>
+  </si>
+  <si>
+    <t>Needs TWS on iMac</t>
+  </si>
+  <si>
+    <t>Install TWS, clone repo</t>
+  </si>
+  <si>
+    <t>PersonalLifeOS</t>
+  </si>
+  <si>
+    <t>SwiftUI habits/schedule</t>
+  </si>
+  <si>
+    <t>Needs clean Xcode build</t>
+  </si>
+  <si>
+    <t>Verify build on MBA, then clone</t>
+  </si>
+  <si>
+    <t>AUTOGIO_PIOS</t>
+  </si>
+  <si>
+    <t>UniFi/Starlink health</t>
+  </si>
+  <si>
+    <t>WAN stability gate reset</t>
+  </si>
+  <si>
+    <t>Re-run WAN gate when on iMac</t>
+  </si>
+  <si>
+    <t>◆ COUNTS</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>◆ CONFIG — Alert Thresholds &amp;amp; Parameters</t>
+  </si>
+  <si>
+    <t>Edit values to change what triggers alerts in the Command Center.</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Liquidity Floor</t>
+  </si>
+  <si>
+    <t>Alert if TOTAL LIQUID &amp;lt; this value</t>
+  </si>
+  <si>
+    <t>Monthly Burn Cap</t>
+  </si>
+  <si>
+    <t>Alert if card spend in any month exceeds this</t>
+  </si>
+  <si>
+    <t>Subscription Stack Cap</t>
+  </si>
+  <si>
+    <t>BRL/mo</t>
+  </si>
+  <si>
+    <t>Alert if total KEEP subscriptions &amp;gt; this</t>
+  </si>
+  <si>
+    <t>Repo Staleness Days</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>Risk score +5 if repo has no commit in this many days</t>
+  </si>
+  <si>
+    <t>FX Rate Low Alert</t>
+  </si>
+  <si>
+    <t>BRL/USD</t>
+  </si>
+  <si>
+    <t>Alert if any FX op below this rate</t>
+  </si>
+  <si>
+    <t>FX Rate High Alert</t>
+  </si>
+  <si>
+    <t>Alert if any FX op above this rate</t>
+  </si>
+  <si>
+    <t>Cancel Savings Target</t>
+  </si>
+  <si>
+    <t>Expected monthly savings from CANCEL queue</t>
+  </si>
+  <si>
+    <t>Renewal Warning Days</t>
+  </si>
+  <si>
+    <t>Alert when a subscription renewal is within this many days</t>
+  </si>
+  <si>
+    <t>Project Stale Days</t>
+  </si>
+  <si>
+    <t>Alert if active project not touched in this many days</t>
+  </si>
+  <si>
+    <t>Net Worth Currency</t>
+  </si>
+  <si>
+    <t>All amounts denominated in BRL unless marked USD</t>
+  </si>
+  <si>
+    <t>Report Period</t>
+  </si>
+  <si>
+    <t>H1 2026</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>CPF redacted</t>
+  </si>
+  <si>
+    <t>◆ MONTHLY — Cash Flow Summary · Jan–Jun 2026</t>
+  </si>
+  <si>
+    <t>One row per month. Card from TRANSACTIONS, PIX from PIX tab, FX from FX_OPS. Update when new month closes.</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Card Spend</t>
+  </si>
+  <si>
+    <t>Txs</t>
+  </si>
+  <si>
+    <t>FX Out</t>
+  </si>
+  <si>
+    <t>FX In</t>
+  </si>
+  <si>
+    <t>Net Flow</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>TOTAL H1 2026</t>
+  </si>
+  <si>
+    <t>AVG/MONTH</t>
+  </si>
+  <si>
+    <t>◆ MoM CHANGES — Card Spend</t>
+  </si>
+  <si>
+    <t>Spend</t>
+  </si>
+  <si>
+    <t>Prior Month</t>
+  </si>
+  <si>
+    <t>MoM %</t>
+  </si>
+  <si>
+    <t>◆ CATEGORIES — Card Spend Breakdown · H1 2026</t>
+  </si>
+  <si>
+    <t>Sorted largest to smallest. Update when full transaction data changes.</t>
+  </si>
+  <si>
+    <t>Total (R$)</t>
+  </si>
+  <si>
+    <t>% of Card</t>
+  </si>
+  <si>
+    <t>Avg/Month</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>💡 Discretionary</t>
+  </si>
+  <si>
+    <t>⚠ Review</t>
+  </si>
+  <si>
+    <t>❓ Unknown</t>
+  </si>
+  <si>
+    <t>✅ Essential</t>
+  </si>
+  <si>
+    <t>Transporte</t>
+  </si>
+  <si>
+    <t>◆ BY CLASSIFICATION</t>
+  </si>
+  <si>
+    <t>◆ ALERTS — Risk &amp;amp; Action Register · Cross-Domain</t>
+  </si>
+  <si>
+    <t>Full alert register. Sources: finance, subscriptions, repos, projects. Update status as resolved.</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Finding</t>
+  </si>
+  <si>
+    <t>BRL Exposure</t>
+  </si>
+  <si>
+    <t>Recommended Action</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
+    <t>Subscriptions</t>
+  </si>
+  <si>
+    <t>CANCEL queue: Claude x2 (R$184/mo) + Grok (R$149.90/mo) + TuneIn (R$31.90/mo) = R$365.80/mo</t>
+  </si>
+  <si>
+    <t>Cancel all 4 before next billing. Apple Subscriptions + app accounts.</t>
+  </si>
+  <si>
+    <t>FX Reconciliation</t>
+  </si>
+  <si>
+    <t>R$652,789 sent to USA Own Account (67995). 19 ops Jan-Jun. Validate USD balances vs BCB.</t>
+  </si>
+  <si>
+    <t>Pull USD account statement. Reconcile each BCB op against balance.</t>
+  </si>
+  <si>
+    <t>Sub Stack Bloat</t>
+  </si>
+  <si>
+    <t>6 services in REVIEW. Annual exposure ~R$7,763. Manus credits uncontrolled.</t>
+  </si>
+  <si>
+    <t>Audit each REVIEW service. Decide KEEP/CANCEL. Target: eliminate ≥3.</t>
+  </si>
+  <si>
+    <t>Liquidity</t>
+  </si>
+  <si>
+    <t>100% liquid in 2 digital banks (Inter + MP = R$23,197). BB balance R$0. Below R$30k target.</t>
+  </si>
+  <si>
+    <t>Maintain R$30k+ buffer. Distribute across BB Rende Fácil + Inter.</t>
+  </si>
+  <si>
+    <t>IOF + FX Cost</t>
+  </si>
+  <si>
+    <t>R$3,475 IOF paid on Inter FX. Compare rates across Wise / Topázio / BB.</t>
+  </si>
+  <si>
+    <t>Review IOF rate per op. Compare institutions for next transfers.</t>
+  </si>
+  <si>
+    <t>IB Withdrawal</t>
+  </si>
+  <si>
+    <t>R$19,196 IB withdrawal via Wise Jun/2026. Destination unconfirmed.</t>
+  </si>
+  <si>
+    <t>Confirm destination. Check Inter + IB statements.</t>
+  </si>
+  <si>
+    <t>Lottery/Gambling</t>
+  </si>
+  <si>
+    <t>R$6,455 Loteria on MP card (39 txs). No budget cap. Avg R$1,076/mo.</t>
+  </si>
+  <si>
+    <t>Set monthly Loteria limit R$500. Remove card if exceeded.</t>
+  </si>
+  <si>
+    <t>AI/Tech Overlap</t>
+  </si>
+  <si>
+    <t>R$6,624 via card on IA/Tech (37 txs). Likely duplicates subscription stack.</t>
+  </si>
+  <si>
+    <t>Cross-match card IA charges vs sub list. Consolidate billing method.</t>
+  </si>
+  <si>
+    <t>Travel/Viagem</t>
+  </si>
+  <si>
+    <t>R$9,037 travel charges (LAN Airlines Mar/2026). Business vs personal unclassified.</t>
+  </si>
+  <si>
+    <t>Classify: business vs personal. Flag deductible items.</t>
+  </si>
+  <si>
+    <t>ML Volume</t>
+  </si>
+  <si>
+    <t>R$31,570 Mercado Livre purchases. Strong Home Office + CPAP pattern. No tags.</t>
+  </si>
+  <si>
+    <t>Tag each purchase: CAPEX / HEALTH / CONSUMABLE for tax tracking.</t>
+  </si>
+  <si>
+    <t>Multiple Wise ops (IB deposits + UK transfers). Ensure BACEN reporting.</t>
+  </si>
+  <si>
+    <t>Confirm BACEN reporting compliance. Keep KYC current.</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>SBCT Tech Solutions</t>
+  </si>
+  <si>
+    <t>R$45,000 PIX Out to SBCT Tech Solutions LLC (USA) via Inter May/2026.</t>
+  </si>
+  <si>
+    <t>Confirm nature: service invoice? investment? Ensure documentation.</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>clean</t>
+  </si>
+  <si>
+    <t>Personal_Finance</t>
+  </si>
+  <si>
+    <t>Wealth + ops dashboards</t>
+  </si>
+  <si>
+    <t>Weekly ops pass: balances + transactions</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>fix/report-accuracy-v1</t>
+  </si>
+  <si>
+    <t>github.com/AUTOGIO/Personal_Finance_Dashboards</t>
+  </si>
+  <si>
+    <t>Wealth + ops dashboards · uncommitted: unfreeze edits</t>
+  </si>
+  <si>
+    <t>Mac system health · clean, on feature branch</t>
   </si>
 </sst>
 </file>
@@ -5725,7 +5755,7 @@
         <v>220</v>
       </c>
       <c r="J5" s="27" t="s">
-        <v>221</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5757,7 +5787,7 @@
         <v>220</v>
       </c>
       <c r="J6" s="27" t="s">
-        <v>221</v>
+        <v>478</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5873,11 +5903,11 @@
         <v>238</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>232</v>
+        <v>219</v>
       </c>
       <c r="I10" s="27"/>
       <c r="J10" s="27" t="s">
-        <v>239</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6001,7 +6031,7 @@
         <v>253</v>
       </c>
       <c r="J14" s="27" t="s">
-        <v>221</v>
+        <v>478</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6161,7 +6191,7 @@
         <v>272</v>
       </c>
       <c r="J19" s="27" t="s">
-        <v>221</v>
+        <v>478</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6188,11 +6218,11 @@
       </c>
       <c r="E23" s="24" t="n">
         <f aca="false">SUMIFS(E5:E19,H5:H19,"CANCEL")</f>
-        <v>365.8</v>
+        <v>784.23</v>
       </c>
       <c r="F23" s="4" t="n">
         <f aca="false">COUNTIF(H5:H19,"CANCEL")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6201,11 +6231,11 @@
       </c>
       <c r="E24" s="24" t="n">
         <f aca="false">SUMIFS(E5:E19,H5:H19,"REVIEW")</f>
-        <v>646.95</v>
+        <v>228.52</v>
       </c>
       <c r="F24" s="4" t="n">
         <f aca="false">COUNTIF(H5:H19,"REVIEW")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6214,7 +6244,7 @@
       </c>
       <c r="E26" s="10" t="n">
         <f aca="false">E23*12</f>
-        <v>4389.6</v>
+        <v>9410.76</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6856,7 +6886,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>325</v>
+        <v>480</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>326</v>
@@ -6865,27 +6895,27 @@
         <v>327</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>328</v>
+        <v>253</v>
       </c>
       <c r="F5" s="33" t="n">
         <f aca="true">IFERROR(TODAY()-DATEVALUE(E5),"")</f>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>329</v>
+        <v>485</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>330</v>
       </c>
       <c r="I5" s="33" t="n">
         <f aca="false">IF(B5="broken",40,IF(B5="dirty",20+D5,0))+IF(C5&lt;&gt;"main",10,0)+IF(F5&gt;30,5,0)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>331</v>
+        <v>486</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6893,20 +6923,20 @@
         <v>332</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>326</v>
+        <v>479</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>327</v>
+        <v>484</v>
       </c>
       <c r="D6" s="32" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>257</v>
+        <v>483</v>
       </c>
       <c r="F6" s="33" t="n">
         <f aca="true">IFERROR(TODAY()-DATEVALUE(E6),"")</f>
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>333</v>
@@ -6916,10 +6946,10 @@
       </c>
       <c r="I6" s="33" t="n">
         <f aca="false">IF(B6="broken",40,IF(B6="dirty",20+D6,0))+IF(C6&lt;&gt;"main",10,0)+IF(F6&gt;30,5,0)</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>335</v>
+        <v>487</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6942,7 +6972,7 @@
       </c>
       <c r="B10" s="4" t="n">
         <f aca="false">COUNTIF(B5:B6,"clean")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6951,7 +6981,7 @@
       </c>
       <c r="B11" s="4" t="n">
         <f aca="false">COUNTIF(B5:B6,"dirty")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7032,22 +7062,22 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>325</v>
+        <v>480</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>229</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>350</v>
+        <v>481</v>
       </c>
       <c r="D5" s="27" t="s">
         <v>351</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>352</v>
+        <v>482</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>328</v>
+        <v>253</v>
       </c>
       <c r="G5" s="27" t="s">
         <v>218</v>
@@ -7070,7 +7100,7 @@
         <v>354</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>257</v>
+        <v>483</v>
       </c>
       <c r="G6" s="27" t="s">
         <v>218</v>

</xml_diff>